<commit_message>
update ValueSet descr 512e6ec6b6fa3a6a29133ba0d279d92105bf18f2
</commit_message>
<xml_diff>
--- a/nr-uniformisation-descriptions/ig/CodeSystem-fr-core-cs-contact-relationship.xlsx
+++ b/nr-uniformisation-descriptions/ig/CodeSystem-fr-core-cs-contact-relationship.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-11T12:08:53+00:00</t>
+    <t>2025-02-11T15:31:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -87,7 +87,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Relationship</t>
+    <t>Relationship type</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>